<commit_message>
feat: \354\213\234\352\263\204\354\227\264 \353\271\204\352\265\220 \353\260\217 \354\206\214\353\223\235\353\263\204 \355\217\211\352\260\200 \354\212\254\353\234\274\354\235\264\353\223\234 \354\266\224\352\260\200, README \354\227\205\353\215\260\354\230\264\355\212\270
</commit_message>
<xml_diff>
--- a/data/NBS167차_부동산정책평가.xlsx
+++ b/data/NBS167차_부동산정책평가.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\WeeklyOpinion\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA7AF332-CF7C-4FBE-B7BA-DE48410580A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C1E2343-AD19-48E4-9670-D46C7023C840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="1845" windowWidth="21600" windowHeight="11295" xr2:uid="{511C9560-6393-4716-96A7-66065B5F1073}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{511C9560-6393-4716-96A7-66065B5F1073}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet20" sheetId="1" r:id="rId1"/>
@@ -1261,17 +1261,6 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>부산/울산/경남</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <rFont val="Malgun Gothic"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
       <t>(146)</t>
     </r>
   </si>
@@ -3225,13 +3214,17 @@
       </rPr>
       <t>케이스탯리서치, 코리아리서치</t>
     </r>
+  </si>
+  <si>
+    <t>부산/울산/경남</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -3308,6 +3301,12 @@
       <sz val="9"/>
       <name val="Batang"/>
       <family val="1"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
       <charset val="129"/>
     </font>
   </fonts>
@@ -3492,7 +3491,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3649,14 +3648,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="7"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3997,158 +3999,158 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="42" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="22.5">
       <c r="A3" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="17.25">
       <c r="A5" s="43" t="s">
+        <v>221</v>
+      </c>
+      <c r="B5" s="44" t="s">
         <v>222</v>
-      </c>
-      <c r="B5" s="44" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="18" thickBot="1">
       <c r="A6" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="B6" s="46" t="s">
         <v>224</v>
-      </c>
-      <c r="B6" s="46" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="16.5">
       <c r="A7" s="47"/>
       <c r="B7" s="16" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="17.25">
       <c r="A8" s="48" t="s">
+        <v>226</v>
+      </c>
+      <c r="B8" s="26" t="s">
         <v>227</v>
-      </c>
-      <c r="B8" s="26" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="17.25" thickBot="1">
       <c r="A9" s="47"/>
       <c r="B9" s="49" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="18" thickBot="1">
       <c r="A10" s="50" t="s">
+        <v>229</v>
+      </c>
+      <c r="B10" s="51" t="s">
         <v>230</v>
-      </c>
-      <c r="B10" s="51" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="18" thickBot="1">
       <c r="A11" s="50" t="s">
+        <v>231</v>
+      </c>
+      <c r="B11" s="51" t="s">
         <v>232</v>
-      </c>
-      <c r="B11" s="51" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="18" thickBot="1">
       <c r="A12" s="50" t="s">
+        <v>233</v>
+      </c>
+      <c r="B12" s="51" t="s">
         <v>234</v>
       </c>
-      <c r="B12" s="51" t="s">
+    </row>
+    <row r="13" spans="1:2" ht="16.5">
+      <c r="A13" s="54" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" ht="16.5">
-      <c r="A13" s="52" t="s">
+      <c r="B13" s="16" t="s">
         <v>236</v>
       </c>
-      <c r="B13" s="16" t="s">
+    </row>
+    <row r="14" spans="1:2" ht="17.25" thickBot="1">
+      <c r="A14" s="54"/>
+      <c r="B14" s="52" t="s">
         <v>237</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="17.25" thickBot="1">
-      <c r="A14" s="52"/>
-      <c r="B14" s="53" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="18" thickBot="1">
       <c r="A15" s="50" t="s">
+        <v>238</v>
+      </c>
+      <c r="B15" s="51" t="s">
         <v>239</v>
       </c>
-      <c r="B15" s="51" t="s">
+    </row>
+    <row r="16" spans="1:2" ht="16.5">
+      <c r="A16" s="54" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" ht="16.5">
-      <c r="A16" s="52" t="s">
+      <c r="B16" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="B16" s="16" t="s">
+    </row>
+    <row r="17" spans="1:11" ht="17.25" thickBot="1">
+      <c r="A17" s="54"/>
+      <c r="B17" s="52" t="s">
         <v>242</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="17.25" thickBot="1">
-      <c r="A17" s="52"/>
-      <c r="B17" s="53" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="18" thickBot="1">
       <c r="A18" s="50" t="s">
+        <v>243</v>
+      </c>
+      <c r="B18" s="51" t="s">
         <v>244</v>
-      </c>
-      <c r="B18" s="51" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="18" thickBot="1">
       <c r="A19" s="50" t="s">
+        <v>245</v>
+      </c>
+      <c r="B19" s="51" t="s">
         <v>246</v>
-      </c>
-      <c r="B19" s="51" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="16.5">
       <c r="A20" s="47"/>
       <c r="B20" s="16" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="16.5">
+      <c r="A21" s="54" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" ht="16.5">
-      <c r="A21" s="52" t="s">
+      <c r="B21" s="26" t="s">
         <v>249</v>
       </c>
-      <c r="B21" s="26" t="s">
+    </row>
+    <row r="22" spans="1:11" ht="16.5">
+      <c r="A22" s="54"/>
+      <c r="B22" s="26" t="s">
         <v>250</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="16.5">
-      <c r="A22" s="52"/>
-      <c r="B22" s="26" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="17.25" thickBot="1">
       <c r="A23" s="47"/>
-      <c r="B23" s="53" t="s">
+      <c r="B23" s="52" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="18" thickBot="1">
+      <c r="A24" s="53" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" ht="18" thickBot="1">
-      <c r="A24" s="54" t="s">
+      <c r="B24" s="51" t="s">
         <v>253</v>
-      </c>
-      <c r="B24" s="51" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -4691,15 +4693,15 @@
         <v>22</v>
       </c>
     </row>
-    <row r="46" spans="1:11">
-      <c r="A46" s="34" t="s">
+    <row r="46" spans="1:11" ht="13.5">
+      <c r="A46" s="55" t="s">
+        <v>254</v>
+      </c>
+      <c r="B46" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="B46" s="23" t="s">
+      <c r="C46" s="23" t="s">
         <v>98</v>
-      </c>
-      <c r="C46" s="23" t="s">
-        <v>99</v>
       </c>
       <c r="D46" s="24" t="s">
         <v>64</v>
@@ -4717,10 +4719,10 @@
         <v>69</v>
       </c>
       <c r="I46" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="J46" s="23" t="s">
         <v>100</v>
-      </c>
-      <c r="J46" s="23" t="s">
-        <v>101</v>
       </c>
       <c r="K46" s="26" t="s">
         <v>22</v>
@@ -4728,13 +4730,13 @@
     </row>
     <row r="47" spans="1:11" ht="13.5" thickBot="1">
       <c r="A47" s="32" t="s">
+        <v>101</v>
+      </c>
+      <c r="B47" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="B47" s="18" t="s">
-        <v>103</v>
-      </c>
       <c r="C47" s="18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D47" s="19" t="s">
         <v>56</v>
@@ -4752,10 +4754,10 @@
         <v>18</v>
       </c>
       <c r="I47" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="J47" s="18" t="s">
         <v>104</v>
-      </c>
-      <c r="J47" s="18" t="s">
-        <v>105</v>
       </c>
       <c r="K47" s="21" t="s">
         <v>22</v>
@@ -4763,13 +4765,13 @@
     </row>
     <row r="48" spans="1:11">
       <c r="A48" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B48" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B48" s="13" t="s">
+      <c r="C48" s="13" t="s">
         <v>107</v>
-      </c>
-      <c r="C48" s="13" t="s">
-        <v>108</v>
       </c>
       <c r="D48" s="14" t="s">
         <v>33</v>
@@ -4778,13 +4780,13 @@
         <v>28</v>
       </c>
       <c r="F48" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G48" s="15" t="s">
         <v>44</v>
       </c>
       <c r="H48" s="13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I48" s="13" t="s">
         <v>34</v>
@@ -4798,13 +4800,13 @@
     </row>
     <row r="49" spans="1:11" ht="19.5">
       <c r="A49" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B49" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="B49" s="23" t="s">
+      <c r="C49" s="23" t="s">
         <v>111</v>
-      </c>
-      <c r="C49" s="23" t="s">
-        <v>112</v>
       </c>
       <c r="D49" s="24" t="s">
         <v>26</v>
@@ -4822,7 +4824,7 @@
         <v>64</v>
       </c>
       <c r="I49" s="23" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J49" s="23" t="s">
         <v>21</v>
@@ -4836,16 +4838,16 @@
         <v>10</v>
       </c>
       <c r="B50" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="C50" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="C50" s="20" t="s">
+      <c r="D50" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D50" s="19" t="s">
+      <c r="E50" s="20" t="s">
         <v>116</v>
-      </c>
-      <c r="E50" s="20" t="s">
-        <v>117</v>
       </c>
       <c r="F50" s="20" t="s">
         <v>19</v>
@@ -4857,7 +4859,7 @@
         <v>42</v>
       </c>
       <c r="I50" s="18" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J50" s="18" t="s">
         <v>18</v>
@@ -4868,19 +4870,19 @@
     </row>
     <row r="51" spans="1:11">
       <c r="A51" s="36" t="s">
+        <v>117</v>
+      </c>
+      <c r="B51" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="B51" s="13" t="s">
+      <c r="C51" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="C51" s="13" t="s">
+      <c r="D51" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="D51" s="15" t="s">
-        <v>121</v>
-      </c>
       <c r="E51" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F51" s="15" t="s">
         <v>20</v>
@@ -4903,13 +4905,13 @@
     </row>
     <row r="52" spans="1:11">
       <c r="A52" s="37" t="s">
+        <v>121</v>
+      </c>
+      <c r="B52" s="28" t="s">
         <v>122</v>
       </c>
-      <c r="B52" s="28" t="s">
+      <c r="C52" s="28" t="s">
         <v>123</v>
-      </c>
-      <c r="C52" s="28" t="s">
-        <v>124</v>
       </c>
       <c r="D52" s="29" t="s">
         <v>26</v>
@@ -4918,7 +4920,7 @@
         <v>48</v>
       </c>
       <c r="F52" s="30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G52" s="30" t="s">
         <v>28</v>
@@ -4938,13 +4940,13 @@
     </row>
     <row r="53" spans="1:11">
       <c r="A53" s="27" t="s">
+        <v>124</v>
+      </c>
+      <c r="B53" s="28" t="s">
         <v>125</v>
       </c>
-      <c r="B53" s="28" t="s">
-        <v>126</v>
-      </c>
       <c r="C53" s="28" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D53" s="29" t="s">
         <v>93</v>
@@ -4962,10 +4964,10 @@
         <v>64</v>
       </c>
       <c r="I53" s="28" t="s">
+        <v>126</v>
+      </c>
+      <c r="J53" s="28" t="s">
         <v>127</v>
-      </c>
-      <c r="J53" s="28" t="s">
-        <v>128</v>
       </c>
       <c r="K53" s="31" t="s">
         <v>22</v>
@@ -4973,13 +4975,13 @@
     </row>
     <row r="54" spans="1:11">
       <c r="A54" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="B54" s="28" t="s">
         <v>129</v>
       </c>
-      <c r="B54" s="28" t="s">
+      <c r="C54" s="28" t="s">
         <v>130</v>
-      </c>
-      <c r="C54" s="28" t="s">
-        <v>131</v>
       </c>
       <c r="D54" s="29" t="s">
         <v>26</v>
@@ -4997,7 +4999,7 @@
         <v>33</v>
       </c>
       <c r="I54" s="28" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J54" s="28" t="s">
         <v>37</v>
@@ -5008,13 +5010,13 @@
     </row>
     <row r="55" spans="1:11">
       <c r="A55" s="27" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B55" s="28" t="s">
         <v>72</v>
       </c>
       <c r="C55" s="28" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D55" s="29" t="s">
         <v>56</v>
@@ -5029,7 +5031,7 @@
         <v>35</v>
       </c>
       <c r="H55" s="28" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I55" s="28" t="s">
         <v>48</v>
@@ -5043,13 +5045,13 @@
     </row>
     <row r="56" spans="1:11">
       <c r="A56" s="27" t="s">
+        <v>134</v>
+      </c>
+      <c r="B56" s="28" t="s">
         <v>135</v>
       </c>
-      <c r="B56" s="28" t="s">
-        <v>136</v>
-      </c>
       <c r="C56" s="28" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D56" s="29" t="s">
         <v>41</v>
@@ -5058,7 +5060,7 @@
         <v>86</v>
       </c>
       <c r="F56" s="30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G56" s="30" t="s">
         <v>19</v>
@@ -5070,7 +5072,7 @@
         <v>27</v>
       </c>
       <c r="J56" s="28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K56" s="31" t="s">
         <v>22</v>
@@ -5078,13 +5080,13 @@
     </row>
     <row r="57" spans="1:11">
       <c r="A57" s="34" t="s">
+        <v>136</v>
+      </c>
+      <c r="B57" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="B57" s="23" t="s">
+      <c r="C57" s="23" t="s">
         <v>138</v>
-      </c>
-      <c r="C57" s="23" t="s">
-        <v>139</v>
       </c>
       <c r="D57" s="24" t="s">
         <v>41</v>
@@ -5116,31 +5118,31 @@
         <v>10</v>
       </c>
       <c r="B58" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="C58" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="C58" s="20" t="s">
-        <v>141</v>
-      </c>
       <c r="D58" s="19" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E58" s="20" t="s">
         <v>81</v>
       </c>
       <c r="F58" s="20" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G58" s="20" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H58" s="18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I58" s="18" t="s">
         <v>81</v>
       </c>
       <c r="J58" s="18" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K58" s="21" t="s">
         <v>22</v>
@@ -5148,13 +5150,13 @@
     </row>
     <row r="59" spans="1:11">
       <c r="A59" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="B59" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="B59" s="13" t="s">
-        <v>144</v>
-      </c>
       <c r="C59" s="13" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D59" s="14" t="s">
         <v>26</v>
@@ -5172,7 +5174,7 @@
         <v>33</v>
       </c>
       <c r="I59" s="13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J59" s="13" t="s">
         <v>45</v>
@@ -5183,22 +5185,22 @@
     </row>
     <row r="60" spans="1:11" ht="19.5">
       <c r="A60" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="B60" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="B60" s="23" t="s">
+      <c r="C60" s="23" t="s">
         <v>146</v>
-      </c>
-      <c r="C60" s="23" t="s">
-        <v>147</v>
       </c>
       <c r="D60" s="24" t="s">
         <v>26</v>
       </c>
       <c r="E60" s="25" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F60" s="25" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G60" s="25" t="s">
         <v>44</v>
@@ -5210,7 +5212,7 @@
         <v>70</v>
       </c>
       <c r="J60" s="23" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K60" s="26" t="s">
         <v>22</v>
@@ -5218,13 +5220,13 @@
     </row>
     <row r="61" spans="1:11" ht="21">
       <c r="A61" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="B61" s="28" t="s">
         <v>148</v>
       </c>
-      <c r="B61" s="28" t="s">
+      <c r="C61" s="28" t="s">
         <v>149</v>
-      </c>
-      <c r="C61" s="28" t="s">
-        <v>150</v>
       </c>
       <c r="D61" s="29" t="s">
         <v>33</v>
@@ -5233,7 +5235,7 @@
         <v>86</v>
       </c>
       <c r="F61" s="30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G61" s="30" t="s">
         <v>55</v>
@@ -5242,7 +5244,7 @@
         <v>61</v>
       </c>
       <c r="I61" s="28" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J61" s="28" t="s">
         <v>29</v>
@@ -5256,16 +5258,16 @@
         <v>10</v>
       </c>
       <c r="B62" s="18" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C62" s="18" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D62" s="19" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E62" s="20" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F62" s="20" t="s">
         <v>54</v>
@@ -5274,10 +5276,10 @@
         <v>26</v>
       </c>
       <c r="H62" s="18" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I62" s="18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J62" s="18" t="s">
         <v>42</v>
@@ -5288,13 +5290,13 @@
     </row>
     <row r="63" spans="1:11">
       <c r="A63" s="36" t="s">
+        <v>152</v>
+      </c>
+      <c r="B63" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="C63" s="13" t="s">
         <v>153</v>
-      </c>
-      <c r="B63" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="C63" s="13" t="s">
-        <v>154</v>
       </c>
       <c r="D63" s="15" t="s">
         <v>61</v>
@@ -5306,7 +5308,7 @@
         <v>55</v>
       </c>
       <c r="G63" s="15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H63" s="13" t="s">
         <v>69</v>
@@ -5323,13 +5325,13 @@
     </row>
     <row r="64" spans="1:11">
       <c r="A64" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="B64" s="28" t="s">
         <v>156</v>
       </c>
-      <c r="B64" s="28" t="s">
+      <c r="C64" s="28" t="s">
         <v>157</v>
-      </c>
-      <c r="C64" s="28" t="s">
-        <v>158</v>
       </c>
       <c r="D64" s="29" t="s">
         <v>74</v>
@@ -5338,10 +5340,10 @@
         <v>69</v>
       </c>
       <c r="F64" s="30" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G64" s="30" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H64" s="28" t="s">
         <v>64</v>
@@ -5350,7 +5352,7 @@
         <v>19</v>
       </c>
       <c r="J64" s="28" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K64" s="31" t="s">
         <v>22</v>
@@ -5358,16 +5360,16 @@
     </row>
     <row r="65" spans="1:11">
       <c r="A65" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="B65" s="23" t="s">
         <v>161</v>
       </c>
-      <c r="B65" s="23" t="s">
+      <c r="C65" s="23" t="s">
         <v>162</v>
       </c>
-      <c r="C65" s="23" t="s">
-        <v>163</v>
-      </c>
       <c r="D65" s="25" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E65" s="25" t="s">
         <v>81</v>
@@ -5379,10 +5381,10 @@
         <v>93</v>
       </c>
       <c r="H65" s="23" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I65" s="23" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J65" s="23" t="s">
         <v>86</v>
@@ -5393,13 +5395,13 @@
     </row>
     <row r="66" spans="1:11" ht="19.5">
       <c r="A66" s="22" t="s">
+        <v>164</v>
+      </c>
+      <c r="B66" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="B66" s="23" t="s">
-        <v>166</v>
-      </c>
       <c r="C66" s="23" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D66" s="24" t="s">
         <v>41</v>
@@ -5411,16 +5413,16 @@
         <v>65</v>
       </c>
       <c r="G66" s="25" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H66" s="23" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I66" s="23" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J66" s="23" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K66" s="26" t="s">
         <v>22</v>
@@ -5428,13 +5430,13 @@
     </row>
     <row r="67" spans="1:11">
       <c r="A67" s="38" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B67" s="25" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C67" s="25" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D67" s="25" t="s">
         <v>19</v>
@@ -5446,13 +5448,13 @@
         <v>42</v>
       </c>
       <c r="G67" s="25" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H67" s="23" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I67" s="23" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J67" s="23" t="s">
         <v>42</v>
@@ -5463,16 +5465,16 @@
     </row>
     <row r="68" spans="1:11">
       <c r="A68" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="B68" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="C68" s="23" t="s">
         <v>170</v>
       </c>
-      <c r="B68" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="C68" s="23" t="s">
-        <v>171</v>
-      </c>
       <c r="D68" s="24" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E68" s="25" t="s">
         <v>18</v>
@@ -5490,7 +5492,7 @@
         <v>18</v>
       </c>
       <c r="J68" s="23" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K68" s="26" t="s">
         <v>22</v>
@@ -5498,22 +5500,22 @@
     </row>
     <row r="69" spans="1:11" ht="13.5" thickBot="1">
       <c r="A69" s="39" t="s">
+        <v>172</v>
+      </c>
+      <c r="B69" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="B69" s="18" t="s">
+      <c r="C69" s="18" t="s">
         <v>174</v>
       </c>
-      <c r="C69" s="18" t="s">
-        <v>175</v>
-      </c>
       <c r="D69" s="19" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E69" s="20" t="s">
         <v>35</v>
       </c>
       <c r="F69" s="20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G69" s="20" t="s">
         <v>48</v>
@@ -5533,16 +5535,16 @@
     </row>
     <row r="70" spans="1:11">
       <c r="A70" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="B70" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="B70" s="13" t="s">
+      <c r="C70" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="C70" s="13" t="s">
-        <v>178</v>
-      </c>
       <c r="D70" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E70" s="15" t="s">
         <v>45</v>
@@ -5557,10 +5559,10 @@
         <v>56</v>
       </c>
       <c r="I70" s="13" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="J70" s="13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K70" s="16" t="s">
         <v>22</v>
@@ -5568,13 +5570,13 @@
     </row>
     <row r="71" spans="1:11">
       <c r="A71" s="27" t="s">
+        <v>179</v>
+      </c>
+      <c r="B71" s="28" t="s">
         <v>180</v>
       </c>
-      <c r="B71" s="28" t="s">
+      <c r="C71" s="28" t="s">
         <v>181</v>
-      </c>
-      <c r="C71" s="28" t="s">
-        <v>182</v>
       </c>
       <c r="D71" s="29" t="s">
         <v>33</v>
@@ -5603,19 +5605,19 @@
     </row>
     <row r="72" spans="1:11" ht="19.5">
       <c r="A72" s="27" t="s">
+        <v>182</v>
+      </c>
+      <c r="B72" s="28" t="s">
+        <v>130</v>
+      </c>
+      <c r="C72" s="28" t="s">
         <v>183</v>
       </c>
-      <c r="B72" s="28" t="s">
-        <v>131</v>
-      </c>
-      <c r="C72" s="28" t="s">
-        <v>184</v>
-      </c>
       <c r="D72" s="29" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E72" s="30" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F72" s="30" t="s">
         <v>96</v>
@@ -5630,7 +5632,7 @@
         <v>75</v>
       </c>
       <c r="J72" s="28" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K72" s="31" t="s">
         <v>22</v>
@@ -5641,13 +5643,13 @@
         <v>10</v>
       </c>
       <c r="B73" s="18" t="s">
+        <v>185</v>
+      </c>
+      <c r="C73" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="C73" s="18" t="s">
-        <v>187</v>
-      </c>
       <c r="D73" s="19" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E73" s="20" t="s">
         <v>75</v>
@@ -5673,13 +5675,13 @@
     </row>
     <row r="74" spans="1:11">
       <c r="A74" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="B74" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="B74" s="13" t="s">
+      <c r="C74" s="13" t="s">
         <v>189</v>
-      </c>
-      <c r="C74" s="13" t="s">
-        <v>190</v>
       </c>
       <c r="D74" s="15" t="s">
         <v>69</v>
@@ -5697,7 +5699,7 @@
         <v>93</v>
       </c>
       <c r="I74" s="13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J74" s="13" t="s">
         <v>42</v>
@@ -5708,13 +5710,13 @@
     </row>
     <row r="75" spans="1:11" ht="19.5">
       <c r="A75" s="22" t="s">
+        <v>190</v>
+      </c>
+      <c r="B75" s="23" t="s">
         <v>191</v>
       </c>
-      <c r="B75" s="23" t="s">
+      <c r="C75" s="23" t="s">
         <v>192</v>
-      </c>
-      <c r="C75" s="23" t="s">
-        <v>193</v>
       </c>
       <c r="D75" s="24" t="s">
         <v>74</v>
@@ -5735,7 +5737,7 @@
         <v>93</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K75" s="26" t="s">
         <v>22</v>
@@ -5755,16 +5757,16 @@
         <v>56</v>
       </c>
       <c r="E76" s="20" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F76" s="20" t="s">
         <v>54</v>
       </c>
       <c r="G76" s="20" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H76" s="18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I76" s="18" t="s">
         <v>35</v>
@@ -5778,19 +5780,19 @@
     </row>
     <row r="77" spans="1:11">
       <c r="A77" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="B77" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="B77" s="13" t="s">
+      <c r="C77" s="13" t="s">
         <v>196</v>
-      </c>
-      <c r="C77" s="13" t="s">
-        <v>197</v>
       </c>
       <c r="D77" s="15" t="s">
         <v>19</v>
       </c>
       <c r="E77" s="15" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F77" s="15" t="s">
         <v>86</v>
@@ -5805,7 +5807,7 @@
         <v>49</v>
       </c>
       <c r="J77" s="13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K77" s="16" t="s">
         <v>22</v>
@@ -5813,13 +5815,13 @@
     </row>
     <row r="78" spans="1:11" ht="19.5">
       <c r="A78" s="22" t="s">
+        <v>198</v>
+      </c>
+      <c r="B78" s="23" t="s">
         <v>199</v>
       </c>
-      <c r="B78" s="23" t="s">
+      <c r="C78" s="23" t="s">
         <v>200</v>
-      </c>
-      <c r="C78" s="23" t="s">
-        <v>201</v>
       </c>
       <c r="D78" s="24" t="s">
         <v>74</v>
@@ -5840,7 +5842,7 @@
         <v>69</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="K78" s="26" t="s">
         <v>22</v>
@@ -5851,10 +5853,10 @@
         <v>10</v>
       </c>
       <c r="B79" s="18" t="s">
+        <v>202</v>
+      </c>
+      <c r="C79" s="18" t="s">
         <v>203</v>
-      </c>
-      <c r="C79" s="18" t="s">
-        <v>204</v>
       </c>
       <c r="D79" s="19" t="s">
         <v>41</v>
@@ -5883,13 +5885,13 @@
     </row>
     <row r="80" spans="1:11">
       <c r="A80" s="12" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B80" s="13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D80" s="14" t="s">
         <v>64</v>
@@ -5904,13 +5906,13 @@
         <v>55</v>
       </c>
       <c r="H80" s="13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I80" s="13" t="s">
         <v>17</v>
       </c>
       <c r="J80" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K80" s="16" t="s">
         <v>22</v>
@@ -5918,13 +5920,13 @@
     </row>
     <row r="81" spans="1:11" ht="19.5">
       <c r="A81" s="22" t="s">
+        <v>205</v>
+      </c>
+      <c r="B81" s="23" t="s">
         <v>206</v>
       </c>
-      <c r="B81" s="23" t="s">
+      <c r="C81" s="23" t="s">
         <v>207</v>
-      </c>
-      <c r="C81" s="23" t="s">
-        <v>208</v>
       </c>
       <c r="D81" s="24" t="s">
         <v>64</v>
@@ -5953,13 +5955,13 @@
     </row>
     <row r="82" spans="1:11">
       <c r="A82" s="40" t="s">
+        <v>208</v>
+      </c>
+      <c r="B82" s="28" t="s">
         <v>209</v>
       </c>
-      <c r="B82" s="28" t="s">
+      <c r="C82" s="28" t="s">
         <v>210</v>
-      </c>
-      <c r="C82" s="28" t="s">
-        <v>211</v>
       </c>
       <c r="D82" s="29" t="s">
         <v>93</v>
@@ -5968,7 +5970,7 @@
         <v>34</v>
       </c>
       <c r="F82" s="30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G82" s="30" t="s">
         <v>55</v>
@@ -5991,31 +5993,31 @@
         <v>10</v>
       </c>
       <c r="B83" s="18" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C83" s="18" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D83" s="19" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E83" s="20" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F83" s="20" t="s">
         <v>42</v>
       </c>
       <c r="G83" s="20" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H83" s="18" t="s">
         <v>20</v>
       </c>
       <c r="I83" s="18" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J83" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K83" s="21" t="s">
         <v>22</v>
@@ -6023,13 +6025,13 @@
     </row>
     <row r="84" spans="1:11" ht="19.5">
       <c r="A84" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="B84" s="13" t="s">
         <v>213</v>
       </c>
-      <c r="B84" s="13" t="s">
+      <c r="C84" s="13" t="s">
         <v>214</v>
-      </c>
-      <c r="C84" s="13" t="s">
-        <v>215</v>
       </c>
       <c r="D84" s="14" t="s">
         <v>33</v>
@@ -6041,7 +6043,7 @@
         <v>48</v>
       </c>
       <c r="G84" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H84" s="13" t="s">
         <v>93</v>
@@ -6050,7 +6052,7 @@
         <v>34</v>
       </c>
       <c r="J84" s="13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="K84" s="16" t="s">
         <v>22</v>
@@ -6058,19 +6060,19 @@
     </row>
     <row r="85" spans="1:11">
       <c r="A85" s="41" t="s">
+        <v>216</v>
+      </c>
+      <c r="B85" s="23" t="s">
         <v>217</v>
       </c>
-      <c r="B85" s="23" t="s">
+      <c r="C85" s="23" t="s">
         <v>218</v>
-      </c>
-      <c r="C85" s="23" t="s">
-        <v>219</v>
       </c>
       <c r="D85" s="24" t="s">
         <v>16</v>
       </c>
       <c r="E85" s="25" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F85" s="25" t="s">
         <v>34</v>
@@ -6096,10 +6098,10 @@
         <v>10</v>
       </c>
       <c r="B86" s="18" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C86" s="18" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D86" s="19" t="s">
         <v>64</v>
@@ -6117,10 +6119,10 @@
         <v>65</v>
       </c>
       <c r="I86" s="18" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J86" s="18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K86" s="21" t="s">
         <v>22</v>
@@ -6137,5 +6139,6 @@
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>